<commit_message>
fix: rename entry_date to order_date in invoice report document
</commit_message>
<xml_diff>
--- a/resources/template/invoice_summary_template.xlsx
+++ b/resources/template/invoice_summary_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\Madyotomo CSV\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mmj\project\PHP\madyotomo\resources\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A75ED2-1B2C-4AB2-A1F2-375B9F5AE7EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96A92F4-E2E0-4798-8315-98B304AB0F4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A3115895-C5D7-4D94-AE88-B92AEE4CC1BC}"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="9960" xr2:uid="{A3115895-C5D7-4D94-AE88-B92AEE4CC1BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -111,10 +111,10 @@
     <t>No. Bukti</t>
   </si>
   <si>
-    <t>[invoice.entry_date]</t>
-  </si>
-  <si>
     <t>[invoice.order_name]</t>
+  </si>
+  <si>
+    <t>[invoice.order_date]</t>
   </si>
 </sst>
 </file>
@@ -122,7 +122,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="_-[$Rp-3809]* #,##0.00_-;\-[$Rp-3809]* #,##0.00_-;_-[$Rp-3809]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-[$Rp-3809]* #,##0.00_-;\-[$Rp-3809]* #,##0.00_-;_-[$Rp-3809]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -238,7 +238,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -248,24 +265,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -285,9 +285,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -325,7 +325,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -431,7 +431,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -573,7 +573,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -593,108 +593,108 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
-        <v>25</v>
+      <c r="A11" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>17</v>
@@ -703,26 +703,26 @@
         <v>18</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="11" t="s">
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="8" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>